<commit_message>
36078 user change- June 4 /2025
</commit_message>
<xml_diff>
--- a/TestData/LV_TMTC0036078_TMTC0036082_VerifyTheMappingOfComplianceAndLegalFieldsFromOpportunityToEngagementCF.xlsx
+++ b/TestData/LV_TMTC0036078_TMTC0036082_VerifyTheMappingOfComplianceAndLegalFieldsFromOpportunityToEngagementCF.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE736FF6-C68A-4A9F-8926-EE81A970BA8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{436A423B-5CD8-4B56-8FCE-FEC304E548D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="708" windowWidth="23256" windowHeight="12456" tabRatio="548" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-23148" yWindow="708" windowWidth="23256" windowHeight="12456" tabRatio="548" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="StandardUsers" sheetId="2" r:id="rId1"/>
@@ -668,13 +668,14 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="9" applyFont="0" applyBorder="0"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyFont="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Accent1 2" xfId="2" xr:uid="{18F405CE-23A4-4C4C-B371-AE456DF50166}"/>
@@ -998,13 +999,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -1012,7 +1013,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -1028,13 +1029,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9FBB8EB1-471A-4668-845A-6810E22F6BA4}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -1042,7 +1043,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>78</v>
       </c>
@@ -1050,7 +1051,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>73</v>
       </c>
@@ -1058,7 +1059,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>75</v>
       </c>
@@ -1074,17 +1075,17 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0293C6CF-D2AF-4FB5-B989-23A4E6860FD2}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1097,22 +1098,22 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D296AE2-31EA-40C7-99FB-9B7E70535054}">
   <dimension ref="A1:A3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>71</v>
       </c>
@@ -1126,15 +1127,15 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AFD13242-055E-41A8-80D8-6F50F1B57F7C}">
   <dimension ref="A1:AE2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="22.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="26.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="26.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>10</v>
       </c>
@@ -1226,14 +1227,14 @@
         <v>38</v>
       </c>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>39</v>
       </c>
       <c r="B2" t="s">
         <v>39</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="4" t="s">
         <v>68</v>
       </c>
       <c r="D2" t="s">
@@ -1331,19 +1332,19 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F2CDCD2-7F5E-40FD-BAB3-4BCEC31CD21E}">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.44140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>56</v>
       </c>
@@ -1369,7 +1370,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>50</v>
       </c>
@@ -1403,13 +1404,13 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F2386AE-B180-4489-BA71-14068DFEFD5A}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="26.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>12</v>
       </c>
@@ -1417,7 +1418,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>68</v>
       </c>
@@ -1437,17 +1438,17 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9447574-C5CB-49C4-BC94-993C1D07E71B}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>76</v>
       </c>

</xml_diff>